<commit_message>
feat(F-NAR-019): TREE-COL-029 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-029.xlsx
+++ b/stories/arbres/TREE-COL-029.xlsx
@@ -2752,17 +2752,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Près de le bac à sable, la poule picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé.</t>
+          <t>Près du bac à sable, la poule picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près de le bac à sable, la &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près du bac à sable, la &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Près de le bac à sable, la &lt;emphasis&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé. [pause]</t>
+          <t>Près du bac à sable, la &lt;emphasis&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>narrateur|Près de le bac à sable, la poule picore autour du ballon.
+          <t>narrateur|Près du bac à sable, la poule picore autour du ballon.
 narrateur|Elle tourne.
 narrateur|Une plume blonde reste dans l'herbe.
 enfant-f|La voix a dit : son œuf est à nous.
@@ -2912,8 +2912,7 @@
 maman|Nous, le nôtre.
 enfant-f|J'ai regardé avant la main.
 narrateur|La poule se recouche, cot cot, rassurée.
-papa|Bravo.
-papa|Tu as vu, puis tu as parlé.</t>
+papa|Tes yeux ont parlé avant ta main.</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
@@ -3133,17 +3132,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>La chèvre pose le nez sur le ballon, près de le bac à sable. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.</t>
+          <t>La chèvre pose le nez sur le ballon, près du bac à sable. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près de le bac à sable. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près du bac à sable. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près de le bac à sable. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près du bac à sable. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3277,7 +3276,7 @@
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre pose le nez sur le ballon, près de le bac à sable.
+          <t>narrateur|La chèvre pose le nez sur le ballon, près du bac à sable.
 narrateur|Sa clochette sonne, courte, un peu rêche.
 enfant-f|La voix a dit : elle ouvre le loquet, c'est drôle.
 narrateur|Sarah voit le loquet, à demi tiré.
@@ -3322,17 +3321,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>La clochette sonne une dernière fois, courte. Le ballon, sablé, repose hors du passage. Le loquet est fermé. J'ai dit, au lieu de rire. Le gilet a perdu son brin de sable. La paille d'or brille encore sur le bois. Le linge rayé ne claque plus. La chèvre mâche, le poil tiède au vent. Le pré redevient large, jusqu'au saule.</t>
+          <t>La clochette sonne une dernière fois, courte. Le ballon, sablé, repose hors du passage. Le loquet est fermé. J'ai dit, au lieu de rire. Le gilet a perdu son brin de sable. La paille d'or brille sur le bois. Le linge rayé ne claque plus. La chèvre mâche, le poil tiède au vent. Le pré redevient large, jusqu'au saule.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La clochette sonne une dernière fois, courte. Le ballon, sablé, repose hors du passage. Le loquet est fermé. J'ai dit, au lieu de rire. Le gilet a perdu son brin de sable. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; brille encore sur le bois. Le linge rayé ne claque plus. La chèvre mâche, le poil tiède au vent. Le pré redevient large, jusqu'au saule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La clochette sonne une dernière fois, courte. Le ballon, sablé, repose hors du passage. Le loquet est fermé. J'ai dit, au lieu de rire. Le gilet a perdu son brin de sable. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; brille sur le bois. Le linge rayé ne claque plus. La chèvre mâche, le poil tiède au vent. Le pré redevient large, jusqu'au saule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La clochette sonne une dernière fois, courte. Le ballon, sablé, repose hors du passage. Le loquet est fermé. J'ai dit, au lieu de rire. Le gilet a perdu son brin de sable. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; brille encore sur le bois. Le linge rayé ne claque plus. La chèvre mâche, le poil tiède au vent. Le pré redevient large, jusqu'au saule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La clochette sonne une dernière fois, courte. Le ballon, sablé, repose hors du passage. Le loquet est fermé. J'ai dit, au lieu de rire. Le gilet a perdu son brin de sable. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; brille sur le bois. Le linge rayé ne claque plus. La chèvre mâche, le poil tiède au vent. Le pré redevient large, jusqu'au saule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3475,7 +3474,7 @@
 enfant-f|Le loquet est fermé.
 enfant-f|J'ai dit, au lieu de rire.
 papa|Le gilet a perdu son brin de sable.
-narrateur|La paille d'or brille encore sur le bois.
+narrateur|La paille d'or brille sur le bois.
 maman|Le linge rayé ne claque plus.
 narrateur|La chèvre mâche, le poil tiède au vent.
 narrateur|Le pré redevient large, jusqu'au saule.</t>
@@ -3510,17 +3509,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le poulain souffle, près de le bac à sable, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.</t>
+          <t>Le poulain souffle, près du bac à sable, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; souffle, près de le bac à sable, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; souffle, près du bac à sable, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; souffle, près de le bac à sable, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet. [pause]</t>
+          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; souffle, près du bac à sable, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3654,7 +3653,7 @@
       </c>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>narrateur|Le poulain souffle, près de le bac à sable, loin du ballon.
+          <t>narrateur|Le poulain souffle, près du bac à sable, loin du ballon.
 narrateur|Sa crinière est en bataille, un peu claire.
 enfant-f|La voix a dit : agite le gilet, il court.
 narrateur|Le gilet claque.
@@ -4277,17 +4276,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>La poule s'approche du seau, près de le bac à sable. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.</t>
+          <t>La poule s'approche du seau, près du bac à sable. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; s'approche du seau, près de le bac à sable. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; s'approche du seau, près du bac à sable. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; s'approche du seau, près de le bac à sable. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main. [pause]</t>
+          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; s'approche du seau, près du bac à sable. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4421,7 +4420,7 @@
       </c>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>narrateur|La poule s'approche du seau, près de le bac à sable.
+          <t>narrateur|La poule s'approche du seau, près du bac à sable.
 narrateur|Elle saute un peu.
 narrateur|Un grain tombe.
 enfant-f|La voix a dit de prendre l'œuf, vite.
@@ -4655,17 +4654,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>La chèvre tire le foin du seau, près de le bac à sable. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe.</t>
+          <t>La chèvre tire le foin du seau, près du bac à sable. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près de le bac à sable. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près du bac à sable. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près de le bac à sable. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près du bac à sable. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4799,7 +4798,7 @@
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre tire le foin du seau, près de le bac à sable.
+          <t>narrateur|La chèvre tire le foin du seau, près du bac à sable.
 narrateur|L'anse penche.
 narrateur|La clochette s'énerve.
 enfant-f|La voix a dit de la laisser sortir.
@@ -4814,8 +4813,7 @@
 narrateur|Sarah pose le seau contre la planche.
 narrateur|La chèvre mange, le poil chaud, rassuré.
 enfant-f|Son dîner, pas la porte.
-papa|Bravo.
-papa|Tu as fermé la phrase, et le loquet.
+papa|La phrase est fermée, et le loquet aussi.
 narrateur|Un brin de foin reste sur sa barbe.</t>
         </is>
       </c>
@@ -5035,17 +5033,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le poulain renifle le seau, près de le bac à sable. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge.</t>
+          <t>Le poulain renifle le seau, près du bac à sable. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; renifle le seau, près de le bac à sable. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; renifle le seau, près du bac à sable. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; renifle le seau, près de le bac à sable. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge. [pause]</t>
+          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; renifle le seau, près du bac à sable. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5179,7 +5177,7 @@
       </c>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>narrateur|Le poulain renifle le seau, près de le bac à sable.
+          <t>narrateur|Le poulain renifle le seau, près du bac à sable.
 narrateur|Le gilet claque au vent.
 narrateur|Il recule.
 enfant-f|La voix a dit de faire peur, pour rire.
@@ -5195,7 +5193,6 @@
 narrateur|Une paille d'or bouge sur sa lèvre.
 enfant-f|J'ai dit le rire.
 enfant-f|Puis je l'ai arrêté.
-papa|Bravo.
 papa|Il mange, sans courir.
 narrateur|Le seau reste, vide, comme une auge.</t>
         </is>
@@ -5805,17 +5802,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>La poule frôle le doudou, près de le bac à sable. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.</t>
+          <t>La poule frôle le doudou, près du bac à sable. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; frôle le doudou, près de le bac à sable. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; frôle le doudou, près du bac à sable. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; frôle le doudou, près de le bac à sable. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd. [pause]</t>
+          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; frôle le doudou, près du bac à sable. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5949,7 +5946,7 @@
       </c>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>narrateur|La poule frôle le doudou, près de le bac à sable.
+          <t>narrateur|La poule frôle le doudou, près du bac à sable.
 narrateur|Elle tire un fil gris, puis recule.
 enfant-f|La voix a dit : cache l'œuf dans le doudou.
 narrateur|Sarah serre le doudou.
@@ -6185,17 +6182,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>La chèvre mâchonne le doudou, près de le bac à sable. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.</t>
+          <t>La chèvre mâchonne le doudou, près du bac à sable. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près de le bac à sable. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près du bac à sable. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près de le bac à sable. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près du bac à sable. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6329,7 +6326,7 @@
       </c>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre mâchonne le doudou, près de le bac à sable.
+          <t>narrateur|La chèvre mâchonne le doudou, près du bac à sable.
 narrateur|Un fil gris pend à sa lèvre.
 enfant-f|Non !
 enfant-f|Il n'est pas à manger !
@@ -6757,17 +6754,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le doudou dort loin des sabots, dans l'herbe. Le poulain a refermé les naseaux, rassasié. Je me suis assise, au lieu de sauter. Le gilet, plié, tient chaud au panier. La paille d'or reste la gardienne du bois. Son souffle a fait un nid invisible. Une oreille grise a un brin, comme une broche. Le bac à sable garde un creux, vide et calme.</t>
+          <t>Le doudou dort loin des sabots, dans l'herbe. Le poulain a refermé les naseaux, rassasié. Je me suis assise, au lieu de sauter. Le gilet, plié, tient chaud au panier. La paille d'or reste la gardienne du bois. Son souffle a fait un nid invisible. Une oreille grise a un brin, comme une broche. Le bac à sable garde un creux, vide et lisse.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou dort loin des sabots, dans l'herbe. Le poulain a refermé les naseaux, rassasié. Je me suis assise, au lieu de sauter. Le gilet, plié, tient chaud au panier. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; reste la gardienne du bois. Son souffle a fait un nid invisible. Une oreille grise a un brin, comme une broche. Le bac à sable garde un creux, vide et calme.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou dort loin des sabots, dans l'herbe. Le poulain a refermé les naseaux, rassasié. Je me suis assise, au lieu de sauter. Le gilet, plié, tient chaud au panier. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; reste la gardienne du bois. Son souffle a fait un nid invisible. Une oreille grise a un brin, comme une broche. Le bac à sable garde un creux, vide et lisse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou dort loin des sabots, dans l'herbe. Le poulain a refermé les naseaux, rassasié. Je me suis assise, au lieu de sauter. Le gilet, plié, tient chaud au panier. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; reste la gardienne du bois. Son souffle a fait un nid invisible. Une oreille grise a un brin, comme une broche. Le bac à sable garde un creux, vide et calme.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou dort loin des sabots, dans l'herbe. Le poulain a refermé les naseaux, rassasié. Je me suis assise, au lieu de sauter. Le gilet, plié, tient chaud au panier. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; reste la gardienne du bois. Son souffle a fait un nid invisible. Une oreille grise a un brin, comme une broche. Le bac à sable garde un creux, vide et lisse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6912,7 +6909,7 @@
 narrateur|La paille d'or reste la gardienne du bois.
 papa|Son souffle a fait un nid invisible.
 narrateur|Une oreille grise a un brin, comme une broche.
-narrateur|Le bac à sable garde un creux, vide et calme.</t>
+narrateur|Le bac à sable garde un creux, vide et lisse.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr">
@@ -8091,17 +8088,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Près de le toboggan, la poule picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé.</t>
+          <t>Près du toboggan, la poule picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près de le toboggan, la &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près du toboggan, la &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Près de le toboggan, la &lt;emphasis&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé. [pause]</t>
+          <t>Près du toboggan, la &lt;emphasis&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8235,7 +8232,7 @@
       </c>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>narrateur|Près de le toboggan, la poule picore autour du ballon.
+          <t>narrateur|Près du toboggan, la poule picore autour du ballon.
 narrateur|Elle tourne.
 narrateur|Une plume blonde reste dans l'herbe.
 enfant-f|La voix a dit : son œuf est à nous.
@@ -8251,8 +8248,7 @@
 maman|Nous, le nôtre.
 enfant-f|J'ai regardé avant la main.
 narrateur|La poule se recouche, cot cot, rassurée.
-papa|Bravo.
-papa|Tu as vu, puis tu as parlé.</t>
+papa|Tes yeux ont parlé avant ta main.</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr">
@@ -8472,17 +8468,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>La chèvre pose le nez sur le ballon, près de le toboggan. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.</t>
+          <t>La chèvre pose le nez sur le ballon, près du toboggan. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près de le toboggan. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près du toboggan. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près de le toboggan. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près du toboggan. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8616,7 +8612,7 @@
       </c>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre pose le nez sur le ballon, près de le toboggan.
+          <t>narrateur|La chèvre pose le nez sur le ballon, près du toboggan.
 narrateur|Sa clochette sonne, courte, un peu rêche.
 enfant-f|La voix a dit : elle ouvre le loquet, c'est drôle.
 narrateur|Sarah voit le loquet, à demi tiré.
@@ -8849,17 +8845,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Le poulain souffle, près de le toboggan, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.</t>
+          <t>Le poulain souffle, près du toboggan, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; souffle, près de le toboggan, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; souffle, près du toboggan, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; souffle, près de le toboggan, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet. [pause]</t>
+          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; souffle, près du toboggan, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8993,7 +8989,7 @@
       </c>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>narrateur|Le poulain souffle, près de le toboggan, loin du ballon.
+          <t>narrateur|Le poulain souffle, près du toboggan, loin du ballon.
 narrateur|Sa crinière est en bataille, un peu claire.
 enfant-f|La voix a dit : agite le gilet, il court.
 narrateur|Le gilet claque.
@@ -9041,17 +9037,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le poulain a quitté l'ombre du toboggan. Le ballon reste au pied, comme une borne. Le gilet est plié. Il ne fait plus peur. Sa crinière est redescendue. La paille d'or accroche le bois, pas le tissu. Tes paumes n'ont plus le piquant du métal. Un brin de foin glisse encore sur la rampe. Le hangar avale le dernier rond de soleil.</t>
+          <t>Le poulain a quitté l'ombre du toboggan. Le ballon reste au pied, comme une borne. Le gilet est plié. Il ne fait plus peur. Sa crinière est redescendue. La paille d'or accroche le bois, pas le tissu. Tes paumes n'ont plus le piquant du métal. Un brin de foin glisse sur la rampe. Le hangar avale le dernier rond de soleil.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le poulain a quitté l'ombre du toboggan. Le ballon reste au pied, comme une borne. Le gilet est plié. Il ne fait plus peur. Sa crinière est redescendue. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; accroche le bois, pas le tissu. Tes paumes n'ont plus le piquant du métal. Un brin de foin glisse encore sur la rampe. Le hangar avale le dernier rond de soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le poulain a quitté l'ombre du toboggan. Le ballon reste au pied, comme une borne. Le gilet est plié. Il ne fait plus peur. Sa crinière est redescendue. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; accroche le bois, pas le tissu. Tes paumes n'ont plus le piquant du métal. Un brin de foin glisse sur la rampe. Le hangar avale le dernier rond de soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le poulain a quitté l'ombre du toboggan. Le ballon reste au pied, comme une borne. Le gilet est plié. Il ne fait plus peur. Sa crinière est redescendue. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; accroche le bois, pas le tissu. Tes paumes n'ont plus le piquant du métal. Un brin de foin glisse encore sur la rampe. Le hangar avale le dernier rond de soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le poulain a quitté l'ombre du toboggan. Le ballon reste au pied, comme une borne. Le gilet est plié. Il ne fait plus peur. Sa crinière est redescendue. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; accroche le bois, pas le tissu. Tes paumes n'ont plus le piquant du métal. Un brin de foin glisse sur la rampe. Le hangar avale le dernier rond de soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9196,7 +9192,7 @@
 papa|Sa crinière est redescendue.
 narrateur|La paille d'or accroche le bois, pas le tissu.
 maman|Tes paumes n'ont plus le piquant du métal.
-narrateur|Un brin de foin glisse encore sur la rampe.
+narrateur|Un brin de foin glisse sur la rampe.
 narrateur|Le hangar avale le dernier rond de soleil.</t>
         </is>
       </c>
@@ -9614,17 +9610,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>La poule s'approche du seau, près de le toboggan. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.</t>
+          <t>La poule s'approche du seau, près du toboggan. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; s'approche du seau, près de le toboggan. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; s'approche du seau, près du toboggan. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; s'approche du seau, près de le toboggan. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main. [pause]</t>
+          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; s'approche du seau, près du toboggan. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9758,7 +9754,7 @@
       </c>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>narrateur|La poule s'approche du seau, près de le toboggan.
+          <t>narrateur|La poule s'approche du seau, près du toboggan.
 narrateur|Elle saute un peu.
 narrateur|Un grain tombe.
 enfant-f|La voix a dit de prendre l'œuf, vite.
@@ -9992,17 +9988,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>La chèvre tire le foin du seau, près de le toboggan. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe.</t>
+          <t>La chèvre tire le foin du seau, près du toboggan. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près de le toboggan. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près du toboggan. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près de le toboggan. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près du toboggan. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10136,7 +10132,7 @@
       </c>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre tire le foin du seau, près de le toboggan.
+          <t>narrateur|La chèvre tire le foin du seau, près du toboggan.
 narrateur|L'anse penche.
 narrateur|La clochette s'énerve.
 enfant-f|La voix a dit de la laisser sortir.
@@ -10151,8 +10147,7 @@
 narrateur|Sarah pose le seau contre la planche.
 narrateur|La chèvre mange, le poil chaud, rassuré.
 enfant-f|Son dîner, pas la porte.
-papa|Bravo.
-papa|Tu as fermé la phrase, et le loquet.
+papa|La phrase est fermée, et le loquet aussi.
 narrateur|Un brin de foin reste sur sa barbe.</t>
         </is>
       </c>
@@ -10373,17 +10368,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le poulain renifle le seau, près de le toboggan. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge.</t>
+          <t>Le poulain renifle le seau, près du toboggan. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; renifle le seau, près de le toboggan. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; renifle le seau, près du toboggan. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; renifle le seau, près de le toboggan. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge. [pause]</t>
+          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; renifle le seau, près du toboggan. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10517,7 +10512,7 @@
       </c>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>narrateur|Le poulain renifle le seau, près de le toboggan.
+          <t>narrateur|Le poulain renifle le seau, près du toboggan.
 narrateur|Le gilet claque au vent.
 narrateur|Il recule.
 enfant-f|La voix a dit de faire peur, pour rire.
@@ -10533,7 +10528,6 @@
 narrateur|Une paille d'or bouge sur sa lèvre.
 enfant-f|J'ai dit le rire.
 enfant-f|Puis je l'ai arrêté.
-papa|Bravo.
 papa|Il mange, sans courir.
 narrateur|Le seau reste, vide, comme une auge.</t>
         </is>
@@ -11140,17 +11134,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>La poule frôle le doudou, près de le toboggan. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.</t>
+          <t>La poule frôle le doudou, près du toboggan. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; frôle le doudou, près de le toboggan. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; frôle le doudou, près du toboggan. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; frôle le doudou, près de le toboggan. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd. [pause]</t>
+          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; frôle le doudou, près du toboggan. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11284,7 +11278,7 @@
       </c>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>narrateur|La poule frôle le doudou, près de le toboggan.
+          <t>narrateur|La poule frôle le doudou, près du toboggan.
 narrateur|Elle tire un fil gris, puis recule.
 enfant-f|La voix a dit : cache l'œuf dans le doudou.
 narrateur|Sarah serre le doudou.
@@ -11518,17 +11512,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>La chèvre mâchonne le doudou, près de le toboggan. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.</t>
+          <t>La chèvre mâchonne le doudou, près du toboggan. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près de le toboggan. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près du toboggan. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près de le toboggan. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près du toboggan. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11662,7 +11656,7 @@
       </c>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre mâchonne le doudou, près de le toboggan.
+          <t>narrateur|La chèvre mâchonne le doudou, près du toboggan.
 narrateur|Un fil gris pend à sa lèvre.
 enfant-f|Non !
 enfant-f|Il n'est pas à manger !
@@ -11712,17 +11706,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a un fil repris, encore un peu humide. La chèvre a échangé le gris contre le foin. J'étais sur la marche. J'ai parlé. Le loquet a entendu, lui aussi. Le gilet n'accroche plus la rampe. La paille d'or garde la barrière. Une clochette, très loin, fait un point d'or. Le toboggan devient gris, comme le doudou.</t>
+          <t>Le doudou a un fil repris, un peu humide. La chèvre a échangé le gris contre le foin. J'étais sur la marche. J'ai parlé. Le loquet a entendu, lui aussi. Le gilet n'accroche plus la rampe. La paille d'or garde la barrière. Une clochette, très loin, fait un point d'or. Le toboggan devient gris, comme le doudou.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a un fil repris, encore un peu humide. La chèvre a échangé le gris contre le foin. J'étais sur la marche. J'ai parlé. Le loquet a entendu, lui aussi. Le gilet n'accroche plus la rampe. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; garde la barrière. Une clochette, très loin, fait un point d'or. Le toboggan devient gris, comme le doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a un fil repris, un peu humide. La chèvre a échangé le gris contre le foin. J'étais sur la marche. J'ai parlé. Le loquet a entendu, lui aussi. Le gilet n'accroche plus la rampe. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; garde la barrière. Une clochette, très loin, fait un point d'or. Le toboggan devient gris, comme le doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a un fil repris, encore un peu humide. La chèvre a échangé le gris contre le foin. J'étais sur la marche. J'ai parlé. Le loquet a entendu, lui aussi. Le gilet n'accroche plus la rampe. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; garde la barrière. Une clochette, très loin, fait un point d'or. Le toboggan devient gris, comme le doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a un fil repris, un peu humide. La chèvre a échangé le gris contre le foin. J'étais sur la marche. J'ai parlé. Le loquet a entendu, lui aussi. Le gilet n'accroche plus la rampe. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; garde la barrière. Une clochette, très loin, fait un point d'or. Le toboggan devient gris, comme le doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11860,7 +11854,7 @@
       </c>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|Le doudou a un fil repris, encore un peu humide.
+          <t>narrateur|Le doudou a un fil repris, un peu humide.
 narrateur|La chèvre a échangé le gris contre le foin.
 enfant-f|J'étais sur la marche.
 enfant-f|J'ai parlé.
@@ -12091,17 +12085,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Le doudou dort au pied du toboggan, loin des sabots. Le poulain a soufflé le foin, puis mangé. Je n'ai pas sauté. Tu t'es assise. Il est venu. Le gilet, plié, tient chaud aux œufs. La paille d'or n'a plus rien à retenir. La rampe garde une trace de poil gris. Le hangar ferme le jour, tout doucement.</t>
+          <t>Le doudou dort au pied du toboggan, loin des sabots. Le poulain a soufflé le foin, puis mangé. Je n'ai pas sauté. Tu t'es assise. Il est venu. Le gilet, plié, tient chaud aux œufs. La paille d'or n'a plus rien à retenir. La rampe garde une trace de poil gris. Le hangar ferme le jour, sans bruit.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou dort au pied du toboggan, loin des sabots. Le poulain a soufflé le foin, puis mangé. Je n'ai pas sauté. Tu t'es assise. Il est venu. Le gilet, plié, tient chaud aux œufs. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; n'a plus rien à retenir. La rampe garde une trace de poil gris. Le hangar ferme le jour, tout doucement.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou dort au pied du toboggan, loin des sabots. Le poulain a soufflé le foin, puis mangé. Je n'ai pas sauté. Tu t'es assise. Il est venu. Le gilet, plié, tient chaud aux œufs. La &lt;emphasis level="moderate"&gt;paille d'or&lt;/emphasis&gt; n'a plus rien à retenir. La rampe garde une trace de poil gris. Le hangar ferme le jour, sans bruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou dort au pied du toboggan, loin des sabots. Le poulain a soufflé le foin, puis mangé. Je n'ai pas sauté. Tu t'es assise. Il est venu. Le gilet, plié, tient chaud aux œufs. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; n'a plus rien à retenir. La rampe garde une trace de poil gris. Le hangar ferme le jour, tout doucement.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou dort au pied du toboggan, loin des sabots. Le poulain a soufflé le foin, puis mangé. Je n'ai pas sauté. Tu t'es assise. Il est venu. Le gilet, plié, tient chaud aux œufs. La &lt;emphasis&gt;paille d'or&lt;/emphasis&gt; n'a plus rien à retenir. La rampe garde une trace de poil gris. Le hangar ferme le jour, sans bruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12247,7 +12241,7 @@
 narrateur|Le gilet, plié, tient chaud aux œufs.
 maman|La paille d'or n'a plus rien à retenir.
 narrateur|La rampe garde une trace de poil gris.
-narrateur|Le hangar ferme le jour, tout doucement.</t>
+narrateur|Le hangar ferme le jour, sans bruit.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
@@ -13425,17 +13419,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Près de les balançoires, la poule picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé.</t>
+          <t>Près des balançoires, la poule picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près de les balançoires, la &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près des balançoires, la &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Près de les balançoires, la &lt;emphasis&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Bravo. Tu as vu, puis tu as parlé. [pause]</t>
+          <t>Près des balançoires, la &lt;emphasis&gt;poule&lt;/emphasis&gt; picore autour du ballon. Elle tourne. Une plume blonde reste dans l'herbe. La voix a dit : son œuf est à nous. Sarah avance la main. Puis elle la retire. Elle se baisse. Elle regarde d'abord. Sous l'aile, un creux tiède, un œuf. On ne prend pas. On pose le foin à côté. Le ballon sert de borne, loin de l'œuf. Elle a son nid. Nous, le nôtre. J'ai regardé avant la main. La poule se recouche, cot cot, rassurée. Tes yeux ont parlé avant ta main. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13569,7 +13563,7 @@
       </c>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>narrateur|Près de les balançoires, la poule picore autour du ballon.
+          <t>narrateur|Près des balançoires, la poule picore autour du ballon.
 narrateur|Elle tourne.
 narrateur|Une plume blonde reste dans l'herbe.
 enfant-f|La voix a dit : son œuf est à nous.
@@ -13585,8 +13579,7 @@
 maman|Nous, le nôtre.
 enfant-f|J'ai regardé avant la main.
 narrateur|La poule se recouche, cot cot, rassurée.
-papa|Bravo.
-papa|Tu as vu, puis tu as parlé.</t>
+papa|Tes yeux ont parlé avant ta main.</t>
         </is>
       </c>
       <c r="AX66" t="inlineStr">
@@ -13807,17 +13800,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>La chèvre pose le nez sur le ballon, près de les balançoires. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.</t>
+          <t>La chèvre pose le nez sur le ballon, près des balançoires. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près de les balançoires. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près des balançoires. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près de les balançoires. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; pose le nez sur le ballon, près des balançoires. Sa clochette sonne, courte, un peu rêche. La voix a dit : elle ouvre le loquet, c'est drôle. Sarah voit le loquet, à demi tiré. Elle n'y touche pas toute seule. Papa, le loquet. La voix voulait que je rie. Moi, je n'ai pas ri. On le referme ensemble, alors. Le ballon roule hors du passage. Le foin, lui, va dans son coin à elle. La chèvre mâche. La clochette se tait. Merci d'avoir dit drôle, et pas drôle. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13951,7 +13944,7 @@
       </c>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre pose le nez sur le ballon, près de les balançoires.
+          <t>narrateur|La chèvre pose le nez sur le ballon, près des balançoires.
 narrateur|Sa clochette sonne, courte, un peu rêche.
 enfant-f|La voix a dit : elle ouvre le loquet, c'est drôle.
 narrateur|Sarah voit le loquet, à demi tiré.
@@ -14185,17 +14178,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Le poulain souffle, près de les balançoires, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.</t>
+          <t>Le poulain souffle, près des balançoires, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; souffle, près de les balançoires, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; souffle, près des balançoires, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; souffle, près de les balançoires, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet. [pause]</t>
+          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; souffle, près des balançoires, loin du ballon. Sa crinière est en bataille, un peu claire. La voix a dit : agite le gilet, il court. Le gilet claque. Le poulain recule. Sarah s'arrête. Elle dégrafe le bouton. Je ne veux pas qu'il ait peur. On le plie, alors. Tout petit. Papa pose le ballon, loin des sabots. Sarah étale le foin, plat, sans le jeter. Le poulain avance. Son nez touche le foin. Il mange. Il ne court plus. Merci d'avoir retiré le gilet. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14329,7 +14322,7 @@
       </c>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>narrateur|Le poulain souffle, près de les balançoires, loin du ballon.
+          <t>narrateur|Le poulain souffle, près des balançoires, loin du ballon.
 narrateur|Sa crinière est en bataille, un peu claire.
 enfant-f|La voix a dit : agite le gilet, il court.
 narrateur|Le gilet claque.
@@ -14951,17 +14944,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>La poule s'approche du seau, près de les balançoires. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.</t>
+          <t>La poule s'approche du seau, près des balançoires. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; s'approche du seau, près de les balançoires. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; s'approche du seau, près des balançoires. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; s'approche du seau, près de les balançoires. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main. [pause]</t>
+          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; s'approche du seau, près des balançoires. Elle saute un peu. Un grain tombe. La voix a dit de prendre l'œuf, vite. Sarah pose le seau. Elle ne plonge pas. Elle compte les plumes, une, deux, trois. Tu regardes. C'est bien. Derrière le seau, un nid bas, un œuf chaud. Le foin va autour, pas dessus. Ils font un croissant de foin, à distance. Son nid à elle. Le nôtre à côté. La poule picore le bord, puis s'installe. Merci d'avoir posé le seau, pas la main. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -15095,7 +15088,7 @@
       </c>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|La poule s'approche du seau, près de les balançoires.
+          <t>narrateur|La poule s'approche du seau, près des balançoires.
 narrateur|Elle saute un peu.
 narrateur|Un grain tombe.
 enfant-f|La voix a dit de prendre l'œuf, vite.
@@ -15330,17 +15323,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>La chèvre tire le foin du seau, près de les balançoires. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe.</t>
+          <t>La chèvre tire le foin du seau, près des balançoires. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près de les balançoires. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près des balançoires. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près de les balançoires. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. Bravo. Tu as fermé la phrase, et le loquet. Un brin de foin reste sur sa barbe. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; tire le foin du seau, près des balançoires. L'anse penche. La clochette s'énerve. La voix a dit de la laisser sortir. Sarah voit le loquet. Elle recule d'un pas. Maman, je n'ouvre pas. Ça me serre. On ferme. On lui donne le foin ici. Papa rabat le loquet. Clic, net. Sarah pose le seau contre la planche. La chèvre mange, le poil chaud, rassuré. Son dîner, pas la porte. La phrase est fermée, et le loquet aussi. Un brin de foin reste sur sa barbe. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15474,7 +15467,7 @@
       </c>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre tire le foin du seau, près de les balançoires.
+          <t>narrateur|La chèvre tire le foin du seau, près des balançoires.
 narrateur|L'anse penche.
 narrateur|La clochette s'énerve.
 enfant-f|La voix a dit de la laisser sortir.
@@ -15489,8 +15482,7 @@
 narrateur|Sarah pose le seau contre la planche.
 narrateur|La chèvre mange, le poil chaud, rassuré.
 enfant-f|Son dîner, pas la porte.
-papa|Bravo.
-papa|Tu as fermé la phrase, et le loquet.
+papa|La phrase est fermée, et le loquet aussi.
 narrateur|Un brin de foin reste sur sa barbe.</t>
         </is>
       </c>
@@ -15710,17 +15702,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le poulain renifle le seau, près de les balançoires. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge.</t>
+          <t>Le poulain renifle le seau, près des balançoires. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; renifle le seau, près de les balançoires. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;poulain&lt;/emphasis&gt; renifle le seau, près des balançoires. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; renifle le seau, près de les balançoires. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Bravo. Il mange, sans courir. Le seau reste, vide, comme une auge. [pause]</t>
+          <t>Le &lt;emphasis&gt;poulain&lt;/emphasis&gt; renifle le seau, près des balançoires. Le gilet claque au vent. Il recule. La voix a dit de faire peur, pour rire. Rire, là, ça me serre. Sarah enlève le gilet. Elle le tend à maman. Je le tiens, plié, contre moi. Papa pose le seau. Le foin dépasse, calme. Le poulain revient. Son souffle est chaud. Il croque. Une paille d'or bouge sur sa lèvre. J'ai dit le rire. Puis je l'ai arrêté. Il mange, sans courir. Le seau reste, vide, comme une auge. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15854,7 +15846,7 @@
       </c>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Le poulain renifle le seau, près de les balançoires.
+          <t>narrateur|Le poulain renifle le seau, près des balançoires.
 narrateur|Le gilet claque au vent.
 narrateur|Il recule.
 enfant-f|La voix a dit de faire peur, pour rire.
@@ -15870,7 +15862,6 @@
 narrateur|Une paille d'or bouge sur sa lèvre.
 enfant-f|J'ai dit le rire.
 enfant-f|Puis je l'ai arrêté.
-papa|Bravo.
 papa|Il mange, sans courir.
 narrateur|Le seau reste, vide, comme une auge.</t>
         </is>
@@ -16478,17 +16469,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>La poule frôle le doudou, près de les balançoires. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.</t>
+          <t>La poule frôle le doudou, près des balançoires. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; frôle le doudou, près de les balançoires. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;poule&lt;/emphasis&gt; frôle le doudou, près des balançoires. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; frôle le doudou, près de les balançoires. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd. [pause]</t>
+          <t>La &lt;emphasis&gt;poule&lt;/emphasis&gt; frôle le doudou, près des balançoires. Elle tire un fil gris, puis recule. La voix a dit : cache l'œuf dans le doudou. Sarah serre le doudou. Son ventre dit non. L'œuf n'est pas à cacher. Elle pose le doudou. Elle se penche. Un nid d'herbe, un œuf, tout près du bois. Le doudou veille, loin des pattes. Le foin fait un mur bas, pour le vent. Je n'ai rien pris. J'ai dit. La poule s'installe. L'œuf reste à elle. On a deux nids, et zéro secret lourd. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16622,7 +16613,7 @@
       </c>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>narrateur|La poule frôle le doudou, près de les balançoires.
+          <t>narrateur|La poule frôle le doudou, près des balançoires.
 narrateur|Elle tire un fil gris, puis recule.
 enfant-f|La voix a dit : cache l'œuf dans le doudou.
 narrateur|Sarah serre le doudou.
@@ -16858,17 +16849,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>La chèvre mâchonne le doudou, près de les balançoires. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.</t>
+          <t>La chèvre mâchonne le doudou, près des balançoires. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près de les balançoires. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près des balançoires. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près de les balançoires. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite. [pause]</t>
+          <t>La &lt;emphasis&gt;chèvre&lt;/emphasis&gt; mâchonne le doudou, près des balançoires. Un fil gris pend à sa lèvre. Non ! Il n'est pas à manger ! Sarah tend la main, trop vite, trop près. Elle s'arrête. Elle appelle. Papa, le doudou. La voix a dit : laisse-la. On échange. Du foin contre le doudou. Maman tend le foin. La chèvre lâche le fil. Sarah reprend le doudou, un peu mouillé. J'ai demandé, au lieu de tirer. Merci. Le loquet, on le vérifie aussi. Clic. La clochette redevient petite. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -17002,7 +16993,7 @@
       </c>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>narrateur|La chèvre mâchonne le doudou, près de les balançoires.
+          <t>narrateur|La chèvre mâchonne le doudou, près des balançoires.
 narrateur|Un fil gris pend à sa lèvre.
 enfant-f|Non !
 enfant-f|Il n'est pas à manger !
@@ -17612,7 +17603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17725,6 +17716,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>